<commit_message>
Reorganizar formatos: Notas y entrevistas, Video→Audiovisual, sin Cartilla, Revista anual ni Recursos para docentes
Recategoriza materiales didácticos, AlimentaMENTE y Los ñandúes de Argentina.
El importador convierte los nombres viejos automáticamente.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Mj5tPsRUKGAYe75iT624ru
</commit_message>
<xml_diff>
--- a/plantilla/vocor-planilla-modelo.xlsx
+++ b/plantilla/vocor-planilla-modelo.xlsx
@@ -556,7 +556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -622,7 +622,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Cartilla</t>
+          <t>Libro</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -644,7 +644,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Entrevista</t>
+          <t>Material didáctico</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -666,12 +666,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Libro</t>
+          <t>Notas y entrevistas</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>CIBICI</t>
+          <t>CICTERRA</t>
         </is>
       </c>
     </row>
@@ -688,12 +688,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Material didáctico</t>
+          <t>Podcast</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>CICTERRA</t>
+          <t>CIECS</t>
         </is>
       </c>
     </row>
@@ -702,12 +702,12 @@
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Nota</t>
+          <t>Publicación de divulgación científica</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>CIECS</t>
+          <t>CIT-UNVM</t>
         </is>
       </c>
     </row>
@@ -716,12 +716,12 @@
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Podcast</t>
+          <t>Redes sociales</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>CIT-UNVM</t>
+          <t>EEA Manfredi</t>
         </is>
       </c>
     </row>
@@ -730,12 +730,12 @@
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Publicación de divulgación científica</t>
+          <t>Revista</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>EEA Manfredi</t>
+          <t>IATE</t>
         </is>
       </c>
     </row>
@@ -744,12 +744,12 @@
       <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Recursos para docentes</t>
+          <t>Sitio Web</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>IATE</t>
+          <t>ICYTAC</t>
         </is>
       </c>
     </row>
@@ -758,82 +758,62 @@
       <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Redes sociales</t>
+          <t>Webinar</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>ICYTAC</t>
+          <t>IDACOR</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr"/>
       <c r="B12" t="inlineStr"/>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Revista</t>
-        </is>
-      </c>
+      <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t>IDACOR</t>
+          <t>IDAS</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr"/>
       <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Revista anual</t>
-        </is>
-      </c>
+      <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
-          <t>IDAS</t>
+          <t>IDEA</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr"/>
       <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Sitio Web</t>
-        </is>
-      </c>
+      <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t>IDEA</t>
+          <t>IDEJUS</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr"/>
       <c r="B15" t="inlineStr"/>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Video</t>
-        </is>
-      </c>
+      <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>IDEJUS</t>
+          <t>IECET</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr"/>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Webinar</t>
-        </is>
-      </c>
+      <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
-          <t>IECET</t>
+          <t>IG</t>
         </is>
       </c>
     </row>
@@ -843,7 +823,7 @@
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
-          <t>IG</t>
+          <t>IMBIV</t>
         </is>
       </c>
     </row>
@@ -853,7 +833,7 @@
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
-          <t>IMBIV</t>
+          <t>INFIQC</t>
         </is>
       </c>
     </row>
@@ -863,7 +843,7 @@
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
-          <t>INFIQC</t>
+          <t>INICSA</t>
         </is>
       </c>
     </row>
@@ -873,7 +853,7 @@
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
-          <t>INICSA</t>
+          <t>UDEA</t>
         </is>
       </c>
     </row>
@@ -882,16 +862,6 @@
       <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
-        <is>
-          <t>UDEA</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr"/>
-      <c r="B22" t="inlineStr"/>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr">
         <is>
           <t>UPC-UNC</t>
         </is>

</xml_diff>

<commit_message>
Quitar formatos Webinar y Redes sociales; recategorizar sus materiales
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Mj5tPsRUKGAYe75iT624ru
</commit_message>
<xml_diff>
--- a/plantilla/vocor-planilla-modelo.xlsx
+++ b/plantilla/vocor-planilla-modelo.xlsx
@@ -716,7 +716,7 @@
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Redes sociales</t>
+          <t>Revista</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -730,7 +730,7 @@
       <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Revista</t>
+          <t>Sitio Web</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -742,11 +742,7 @@
     <row r="10">
       <c r="A10" t="inlineStr"/>
       <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Sitio Web</t>
-        </is>
-      </c>
+      <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
           <t>ICYTAC</t>
@@ -756,11 +752,7 @@
     <row r="11">
       <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Webinar</t>
-        </is>
-      </c>
+      <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
           <t>IDACOR</t>

</xml_diff>

<commit_message>
Quitar formato Publicación de divulgación científica: ¿Esto se come? a Libro, Germinación de especies nativas a Material didáctico
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Mj5tPsRUKGAYe75iT624ru
</commit_message>
<xml_diff>
--- a/plantilla/vocor-planilla-modelo.xlsx
+++ b/plantilla/vocor-planilla-modelo.xlsx
@@ -702,7 +702,7 @@
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Publicación de divulgación científica</t>
+          <t>Revista</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -716,7 +716,7 @@
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Revista</t>
+          <t>Sitio Web</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -728,11 +728,7 @@
     <row r="9">
       <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Sitio Web</t>
-        </is>
-      </c>
+      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
           <t>IATE</t>

</xml_diff>

<commit_message>
Planilla modelo: nuevo ejemplo y lista de UE actualizada
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Mj5tPsRUKGAYe75iT624ru
</commit_message>
<xml_diff>
--- a/plantilla/vocor-planilla-modelo.xlsx
+++ b/plantilla/vocor-planilla-modelo.xlsx
@@ -501,12 +501,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Ejemplo: Bichólogos (borrá esta fila)</t>
+          <t>Ejemplo: Plantas nativas de las Sierras (borrá esta fila)</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>IDAS; IMBIV</t>
+          <t>IMBIV; IDEA</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -526,12 +526,12 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>microbios, bacterias</t>
+          <t>plantas nativas, flora, sierras</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Podcast sobre el mundo microbiano.</t>
+          <t>Podcast sobre la flora nativa de Córdoba.</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -556,7 +556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -605,7 +605,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Asociación Argentina de Microbiología Filial Córdoba</t>
+          <t>CCT Cordoba</t>
         </is>
       </c>
     </row>
@@ -627,7 +627,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>CCT Cordoba</t>
+          <t>CEVE</t>
         </is>
       </c>
     </row>
@@ -649,7 +649,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>CEVE</t>
+          <t>CICTERRA</t>
         </is>
       </c>
     </row>
@@ -671,7 +671,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>CICTERRA</t>
+          <t>CIECS</t>
         </is>
       </c>
     </row>
@@ -693,7 +693,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>CIECS</t>
+          <t>CIT-UNVM</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>CIT-UNVM</t>
+          <t>EEA Manfredi</t>
         </is>
       </c>
     </row>
@@ -721,7 +721,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>EEA Manfredi</t>
+          <t>IATE</t>
         </is>
       </c>
     </row>
@@ -731,7 +731,7 @@
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>IATE</t>
+          <t>ICYTAC</t>
         </is>
       </c>
     </row>
@@ -741,7 +741,7 @@
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>ICYTAC</t>
+          <t>IDACOR</t>
         </is>
       </c>
     </row>
@@ -751,7 +751,7 @@
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>IDACOR</t>
+          <t>IDAS</t>
         </is>
       </c>
     </row>
@@ -761,7 +761,7 @@
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t>IDAS</t>
+          <t>IDEA</t>
         </is>
       </c>
     </row>
@@ -771,7 +771,7 @@
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
-          <t>IDEA</t>
+          <t>IDEJUS</t>
         </is>
       </c>
     </row>
@@ -781,7 +781,7 @@
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t>IDEJUS</t>
+          <t>IECET</t>
         </is>
       </c>
     </row>
@@ -791,7 +791,7 @@
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>IECET</t>
+          <t>IG</t>
         </is>
       </c>
     </row>
@@ -801,7 +801,7 @@
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
-          <t>IG</t>
+          <t>IMBIV</t>
         </is>
       </c>
     </row>
@@ -811,7 +811,7 @@
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
-          <t>IMBIV</t>
+          <t>INFIQC</t>
         </is>
       </c>
     </row>
@@ -821,7 +821,7 @@
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
-          <t>INFIQC</t>
+          <t>INICSA</t>
         </is>
       </c>
     </row>
@@ -831,7 +831,7 @@
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
-          <t>INICSA</t>
+          <t>UDEA</t>
         </is>
       </c>
     </row>
@@ -840,16 +840,6 @@
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
-        <is>
-          <t>UDEA</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr"/>
-      <c r="B21" t="inlineStr"/>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr">
         <is>
           <t>UPC-UNC</t>
         </is>

</xml_diff>

<commit_message>
Orden fijo de formatos: Audiovisual, Podcast, Material didáctico, Libro, Revista, Notas y entrevistas, Sitio Web
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Mj5tPsRUKGAYe75iT624ru
</commit_message>
<xml_diff>
--- a/plantilla/vocor-planilla-modelo.xlsx
+++ b/plantilla/vocor-planilla-modelo.xlsx
@@ -622,7 +622,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Libro</t>
+          <t>Podcast</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -666,7 +666,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Notas y entrevistas</t>
+          <t>Libro</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -688,7 +688,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Podcast</t>
+          <t>Revista</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -702,7 +702,7 @@
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Revista</t>
+          <t>Notas y entrevistas</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">

</xml_diff>

<commit_message>
Áreas de materiales unificadas con las de redes; botón "Ver" en la ficha
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Mj5tPsRUKGAYe75iT624ru
</commit_message>
<xml_diff>
--- a/plantilla/vocor-planilla-modelo.xlsx
+++ b/plantilla/vocor-planilla-modelo.xlsx
@@ -556,7 +556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -590,7 +590,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Ciencias Agrarias</t>
+          <t>Ciencias Agrarias, de las Ingenierías y Materiales / Desarrollo Tecnológico y Social</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -605,7 +605,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>CCT Cordoba</t>
+          <t>CEVE</t>
         </is>
       </c>
     </row>
@@ -627,7 +627,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>CEVE</t>
+          <t>CICTERRA</t>
         </is>
       </c>
     </row>
@@ -649,7 +649,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>CICTERRA</t>
+          <t>CIECS</t>
         </is>
       </c>
     </row>
@@ -671,16 +671,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>CIECS</t>
+          <t>CINTRA</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Tecnología, de la Ingeniería y Materiales</t>
-        </is>
-      </c>
+      <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
           <t>Docentes</t>
@@ -707,7 +703,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>EEA Manfredi</t>
+          <t>CITeQ</t>
         </is>
       </c>
     </row>
@@ -721,7 +717,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>IATE</t>
+          <t>EEA Manfredi</t>
         </is>
       </c>
     </row>
@@ -731,7 +727,7 @@
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>ICYTAC</t>
+          <t>IATE</t>
         </is>
       </c>
     </row>
@@ -741,7 +737,7 @@
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>IDACOR</t>
+          <t>ICYTAC</t>
         </is>
       </c>
     </row>
@@ -751,7 +747,7 @@
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>IDAS</t>
+          <t>IDACOR</t>
         </is>
       </c>
     </row>
@@ -761,7 +757,7 @@
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t>IDEA</t>
+          <t>IDAS</t>
         </is>
       </c>
     </row>
@@ -771,7 +767,7 @@
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
-          <t>IDEJUS</t>
+          <t>IDEA</t>
         </is>
       </c>
     </row>
@@ -781,7 +777,7 @@
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t>IECET</t>
+          <t>IDEJUS</t>
         </is>
       </c>
     </row>
@@ -791,7 +787,7 @@
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>IG</t>
+          <t>IDH</t>
         </is>
       </c>
     </row>
@@ -801,7 +797,7 @@
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
-          <t>IMBIV</t>
+          <t>IDIT</t>
         </is>
       </c>
     </row>
@@ -811,7 +807,7 @@
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
-          <t>INFIQC</t>
+          <t>IECET</t>
         </is>
       </c>
     </row>
@@ -821,7 +817,7 @@
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
-          <t>INICSA</t>
+          <t>IEH</t>
         </is>
       </c>
     </row>
@@ -831,7 +827,7 @@
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
-          <t>UDEA</t>
+          <t>IFEC</t>
         </is>
       </c>
     </row>
@@ -840,6 +836,86 @@
       <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
+        <is>
+          <t>IIBYT</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr"/>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>IIPSI</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr"/>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>IMBIV</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr"/>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>INFIQC</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr"/>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>INICSA</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr"/>
+      <c r="B25" t="inlineStr"/>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>ISTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr"/>
+      <c r="B26" t="inlineStr"/>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>UDEA</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr"/>
+      <c r="B27" t="inlineStr"/>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>UNITEFA</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr"/>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr">
         <is>
           <t>UPC-UNC</t>
         </is>

</xml_diff>

<commit_message>
Formato: 'Sitio web'; campo 'oculto' para materiales; Análisis político pasa a Podcast; se ocultan Revista del Museo de Antropología y Del IMBIV para la Comunidad
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Mj5tPsRUKGAYe75iT624ru
</commit_message>
<xml_diff>
--- a/plantilla/vocor-planilla-modelo.xlsx
+++ b/plantilla/vocor-planilla-modelo.xlsx
@@ -556,7 +556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D28"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -712,12 +712,12 @@
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Sitio Web</t>
+          <t>Sitio web</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>EEA Manfredi</t>
+          <t>IATE</t>
         </is>
       </c>
     </row>
@@ -727,7 +727,7 @@
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>IATE</t>
+          <t>ICYTAC</t>
         </is>
       </c>
     </row>
@@ -737,7 +737,7 @@
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>ICYTAC</t>
+          <t>IDACOR</t>
         </is>
       </c>
     </row>
@@ -747,7 +747,7 @@
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>IDACOR</t>
+          <t>IDAS</t>
         </is>
       </c>
     </row>
@@ -757,7 +757,7 @@
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t>IDAS</t>
+          <t>IDEA</t>
         </is>
       </c>
     </row>
@@ -767,7 +767,7 @@
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
-          <t>IDEA</t>
+          <t>IDEJUS</t>
         </is>
       </c>
     </row>
@@ -777,7 +777,7 @@
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t>IDEJUS</t>
+          <t>IDH</t>
         </is>
       </c>
     </row>
@@ -787,7 +787,7 @@
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>IDH</t>
+          <t>IDIT</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
-          <t>IDIT</t>
+          <t>IECET</t>
         </is>
       </c>
     </row>
@@ -807,7 +807,7 @@
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
-          <t>IECET</t>
+          <t>IEH</t>
         </is>
       </c>
     </row>
@@ -817,7 +817,7 @@
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
-          <t>IEH</t>
+          <t>IFEC</t>
         </is>
       </c>
     </row>
@@ -827,7 +827,7 @@
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
-          <t>IFEC</t>
+          <t>IIBYT</t>
         </is>
       </c>
     </row>
@@ -837,7 +837,7 @@
       <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
-          <t>IIBYT</t>
+          <t>IIPSI</t>
         </is>
       </c>
     </row>
@@ -847,7 +847,7 @@
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
-          <t>IIPSI</t>
+          <t>IITEMA</t>
         </is>
       </c>
     </row>
@@ -887,7 +887,7 @@
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
-          <t>ISTE</t>
+          <t>INTA EEA Manfredi</t>
         </is>
       </c>
     </row>
@@ -897,7 +897,7 @@
       <c r="C26" t="inlineStr"/>
       <c r="D26" t="inlineStr">
         <is>
-          <t>UDEA</t>
+          <t>ISTE</t>
         </is>
       </c>
     </row>
@@ -907,7 +907,7 @@
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr">
         <is>
-          <t>UNITEFA</t>
+          <t>UDEA</t>
         </is>
       </c>
     </row>
@@ -916,6 +916,16 @@
       <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr">
+        <is>
+          <t>UNITEFA</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr"/>
+      <c r="B29" t="inlineStr"/>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr">
         <is>
           <t>UPC-UNC</t>
         </is>

</xml_diff>

<commit_message>
Nuevo formato 'En los medios' (reemplaza a Notas y entrevistas, ahora visible)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Mj5tPsRUKGAYe75iT624ru
</commit_message>
<xml_diff>
--- a/plantilla/vocor-planilla-modelo.xlsx
+++ b/plantilla/vocor-planilla-modelo.xlsx
@@ -698,7 +698,7 @@
       <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Notas y entrevistas</t>
+          <t>Sitio web</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -712,7 +712,7 @@
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Sitio web</t>
+          <t>En los medios</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">

</xml_diff>